<commit_message>
looking at vGRF flows
</commit_message>
<xml_diff>
--- a/results/samplewalking/sample/pred_peaks.xlsx
+++ b/results/samplewalking/sample/pred_peaks.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C291"/>
+  <dimension ref="A1:C288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.04377818107605</v>
+        <v>1.224858999252319</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.016365766525269</v>
+        <v>1.057471990585327</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.009666800498962</v>
+        <v>0.9894868135452271</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.043200969696045</v>
+        <v>1.001586198806763</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.090583562850952</v>
+        <v>1.027217268943787</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.103411912918091</v>
+        <v>1.090142369270325</v>
       </c>
     </row>
     <row r="8">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.114682078361511</v>
+        <v>1.081265568733215</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.340420484542847</v>
+        <v>1.209819674491882</v>
       </c>
     </row>
     <row r="10">
@@ -559,7 +559,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1.307485103607178</v>
+        <v>1.322609424591064</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1.153678178787231</v>
+        <v>1.159303188323975</v>
       </c>
     </row>
     <row r="12">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.160569667816162</v>
+        <v>1.089538335800171</v>
       </c>
     </row>
     <row r="13">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.10493278503418</v>
+        <v>1.056803464889526</v>
       </c>
     </row>
     <row r="14">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.141137599945068</v>
+        <v>1.046609997749329</v>
       </c>
     </row>
     <row r="15">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.124887228012085</v>
+        <v>1.219356536865234</v>
       </c>
     </row>
     <row r="16">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1.270630598068237</v>
+        <v>1.050339221954346</v>
       </c>
     </row>
     <row r="17">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.108441829681396</v>
+        <v>1.03770899772644</v>
       </c>
     </row>
     <row r="18">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.085215091705322</v>
+        <v>1.0727698802948</v>
       </c>
     </row>
     <row r="19">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.188253164291382</v>
+        <v>1.053542256355286</v>
       </c>
     </row>
     <row r="20">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.221832871437073</v>
+        <v>1.046705603599548</v>
       </c>
     </row>
     <row r="21">
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.202747941017151</v>
+        <v>1.083330869674683</v>
       </c>
     </row>
     <row r="22">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1.212119340896606</v>
+        <v>1.152071595191956</v>
       </c>
     </row>
     <row r="23">
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.088743209838867</v>
+        <v>1.079880952835083</v>
       </c>
     </row>
     <row r="24">
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1.051110148429871</v>
+        <v>1.300639152526855</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.9916826486587524</v>
+        <v>1.123538732528687</v>
       </c>
     </row>
     <row r="26">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.101776361465454</v>
+        <v>0.9459987878799438</v>
       </c>
     </row>
     <row r="27">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1.103093028068542</v>
+        <v>1.142100095748901</v>
       </c>
     </row>
     <row r="28">
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1.108125329017639</v>
+        <v>0.9863715171813965</v>
       </c>
     </row>
     <row r="29">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1.051948428153992</v>
+        <v>0.9869442582130432</v>
       </c>
     </row>
     <row r="30">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1.391699314117432</v>
+        <v>1.101384162902832</v>
       </c>
     </row>
     <row r="31">
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1.229470372200012</v>
+        <v>1.051348090171814</v>
       </c>
     </row>
     <row r="32">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1.114266872406006</v>
+        <v>1.457407355308533</v>
       </c>
     </row>
     <row r="33">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.146230220794678</v>
+        <v>1.217121124267578</v>
       </c>
     </row>
     <row r="34">
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1.178318500518799</v>
+        <v>1.280094385147095</v>
       </c>
     </row>
     <row r="35">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1.329899549484253</v>
+        <v>1.231905341148376</v>
       </c>
     </row>
     <row r="36">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1.158782005310059</v>
+        <v>1.127145767211914</v>
       </c>
     </row>
     <row r="37">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1.186147928237915</v>
+        <v>1.218099594116211</v>
       </c>
     </row>
     <row r="38">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.069582104682922</v>
+        <v>1.260521173477173</v>
       </c>
     </row>
     <row r="39">
@@ -936,7 +936,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1.085692644119263</v>
+        <v>1.081690311431885</v>
       </c>
     </row>
     <row r="40">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1.199859142303467</v>
+        <v>1.108434319496155</v>
       </c>
     </row>
     <row r="41">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1.123632550239563</v>
+        <v>1.094069123268127</v>
       </c>
     </row>
     <row r="42">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1.063924193382263</v>
+        <v>1.305798053741455</v>
       </c>
     </row>
     <row r="43">
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1.132936716079712</v>
+        <v>1.309473037719727</v>
       </c>
     </row>
     <row r="44">
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.134401321411133</v>
+        <v>1.217161655426025</v>
       </c>
     </row>
     <row r="45">
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1.182366967201233</v>
+        <v>1.087539792060852</v>
       </c>
     </row>
     <row r="46">
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1.097036123275757</v>
+        <v>1.04991602897644</v>
       </c>
     </row>
     <row r="47">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1.128341674804688</v>
+        <v>1.085580587387085</v>
       </c>
     </row>
     <row r="48">
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1.070500731468201</v>
+        <v>1.225558757781982</v>
       </c>
     </row>
     <row r="49">
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1.128471493721008</v>
+        <v>1.082197666168213</v>
       </c>
     </row>
     <row r="50">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1.3625168800354</v>
+        <v>1.069006323814392</v>
       </c>
     </row>
     <row r="51">
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1.221824169158936</v>
+        <v>1.334358096122742</v>
       </c>
     </row>
     <row r="52">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1.041381478309631</v>
+        <v>1.22770631313324</v>
       </c>
     </row>
     <row r="53">
@@ -1118,7 +1118,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1.11417555809021</v>
+        <v>1.042098045349121</v>
       </c>
     </row>
     <row r="54">
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1.040847778320312</v>
+        <v>1.059127569198608</v>
       </c>
     </row>
     <row r="55">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1.256433248519897</v>
+        <v>1.170146346092224</v>
       </c>
     </row>
     <row r="56">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1.173879146575928</v>
+        <v>1.088863849639893</v>
       </c>
     </row>
     <row r="57">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1.140798807144165</v>
+        <v>1.110274791717529</v>
       </c>
     </row>
     <row r="58">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1.276853084564209</v>
+        <v>1.179738521575928</v>
       </c>
     </row>
     <row r="59">
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1.144490718841553</v>
+        <v>1.041194200515747</v>
       </c>
     </row>
     <row r="60">
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1.095381021499634</v>
+        <v>1.197188138961792</v>
       </c>
     </row>
     <row r="61">
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1.150246381759644</v>
+        <v>1.119708299636841</v>
       </c>
     </row>
     <row r="62">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1.188333511352539</v>
+        <v>1.122880458831787</v>
       </c>
     </row>
     <row r="63">
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1.258744955062866</v>
+        <v>1.235860586166382</v>
       </c>
     </row>
     <row r="64">
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.110400199890137</v>
+        <v>1.118414759635925</v>
       </c>
     </row>
     <row r="65">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1.056307911872864</v>
+        <v>1.204912543296814</v>
       </c>
     </row>
     <row r="66">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1.116909980773926</v>
+        <v>1.108945846557617</v>
       </c>
     </row>
     <row r="67">
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1.155988216400146</v>
+        <v>1.298300743103027</v>
       </c>
     </row>
     <row r="68">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1.211126923561096</v>
+        <v>1.326459050178528</v>
       </c>
     </row>
     <row r="69">
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1.065013408660889</v>
+        <v>1.00358521938324</v>
       </c>
     </row>
     <row r="70">
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1.303942203521729</v>
+        <v>1.06489884853363</v>
       </c>
     </row>
     <row r="71">
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1.140904903411865</v>
+        <v>1.310586810112</v>
       </c>
     </row>
     <row r="72">
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.143359184265137</v>
+        <v>1.088800430297852</v>
       </c>
     </row>
     <row r="73">
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.9872176647186279</v>
+        <v>1.353573322296143</v>
       </c>
     </row>
     <row r="74">
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1.126877307891846</v>
+        <v>1.174869775772095</v>
       </c>
     </row>
     <row r="75">
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1.078705668449402</v>
+        <v>1.173592567443848</v>
       </c>
     </row>
     <row r="76">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1.16211462020874</v>
+        <v>1.070054173469543</v>
       </c>
     </row>
     <row r="77">
@@ -1430,7 +1430,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1.286280751228333</v>
+        <v>1.193812370300293</v>
       </c>
     </row>
     <row r="78">
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1.080088257789612</v>
+        <v>1.094552516937256</v>
       </c>
     </row>
     <row r="79">
@@ -1456,7 +1456,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1.119856119155884</v>
+        <v>1.095239162445068</v>
       </c>
     </row>
     <row r="80">
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1.134605050086975</v>
+        <v>1.018330931663513</v>
       </c>
     </row>
     <row r="81">
@@ -1482,7 +1482,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1.176982641220093</v>
+        <v>1.209616541862488</v>
       </c>
     </row>
     <row r="82">
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1.227077960968018</v>
+        <v>1.069148302078247</v>
       </c>
     </row>
     <row r="83">
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.308266282081604</v>
+        <v>1.170395135879517</v>
       </c>
     </row>
     <row r="84">
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1.157287359237671</v>
+        <v>1.168732166290283</v>
       </c>
     </row>
     <row r="85">
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1.173553943634033</v>
+        <v>1.478812098503113</v>
       </c>
     </row>
     <row r="86">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1.110304117202759</v>
+        <v>1.157087564468384</v>
       </c>
     </row>
     <row r="87">
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.152453422546387</v>
+        <v>1.111090898513794</v>
       </c>
     </row>
     <row r="88">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1.232855916023254</v>
+        <v>1.014122247695923</v>
       </c>
     </row>
     <row r="89">
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1.132544755935669</v>
+        <v>1.225677967071533</v>
       </c>
     </row>
     <row r="90">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1.297270655632019</v>
+        <v>1.250590801239014</v>
       </c>
     </row>
     <row r="91">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1.244924068450928</v>
+        <v>1.066640019416809</v>
       </c>
     </row>
     <row r="92">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1.114323139190674</v>
+        <v>1.054853796958923</v>
       </c>
     </row>
     <row r="93">
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1.06743323802948</v>
+        <v>1.138301610946655</v>
       </c>
     </row>
     <row r="94">
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1.202567577362061</v>
+        <v>1.188903093338013</v>
       </c>
     </row>
     <row r="95">
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1.20328962802887</v>
+        <v>1.174735069274902</v>
       </c>
     </row>
     <row r="96">
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1.05058479309082</v>
+        <v>1.098272204399109</v>
       </c>
     </row>
     <row r="97">
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1.092645287513733</v>
+        <v>1.218975901603699</v>
       </c>
     </row>
     <row r="98">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1.062047481536865</v>
+        <v>1.082669496536255</v>
       </c>
     </row>
     <row r="99">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1.120301008224487</v>
+        <v>1.082256078720093</v>
       </c>
     </row>
     <row r="100">
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1.25694739818573</v>
+        <v>1.045490980148315</v>
       </c>
     </row>
     <row r="101">
@@ -1742,7 +1742,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1.086778163909912</v>
+        <v>1.242361903190613</v>
       </c>
     </row>
     <row r="102">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1.221585035324097</v>
+        <v>1.245407819747925</v>
       </c>
     </row>
     <row r="103">
@@ -1768,7 +1768,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1.095352172851562</v>
+        <v>1.208885669708252</v>
       </c>
     </row>
     <row r="104">
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1.163640379905701</v>
+        <v>1.067710280418396</v>
       </c>
     </row>
     <row r="105">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1.245330810546875</v>
+        <v>1.018404960632324</v>
       </c>
     </row>
     <row r="106">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1.070635199546814</v>
+        <v>1.158413648605347</v>
       </c>
     </row>
     <row r="107">
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1.069753646850586</v>
+        <v>1.033069729804993</v>
       </c>
     </row>
     <row r="108">
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1.113839030265808</v>
+        <v>1.066893458366394</v>
       </c>
     </row>
     <row r="109">
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1.061187028884888</v>
+        <v>1.202278971672058</v>
       </c>
     </row>
     <row r="110">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1.141553997993469</v>
+        <v>1.390462398529053</v>
       </c>
     </row>
     <row r="111">
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1.133500099182129</v>
+        <v>0.9989758729934692</v>
       </c>
     </row>
     <row r="112">
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1.142439365386963</v>
+        <v>1.03672182559967</v>
       </c>
     </row>
     <row r="113">
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1.283350706100464</v>
+        <v>1.39847993850708</v>
       </c>
     </row>
     <row r="114">
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1.176900744438171</v>
+        <v>1.376318097114563</v>
       </c>
     </row>
     <row r="115">
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.219615459442139</v>
+        <v>1.214684247970581</v>
       </c>
     </row>
     <row r="116">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1.052890539169312</v>
+        <v>1.325639843940735</v>
       </c>
     </row>
     <row r="117">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1.061892032623291</v>
+        <v>1.098839044570923</v>
       </c>
     </row>
     <row r="118">
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1.134514808654785</v>
+        <v>1.401120901107788</v>
       </c>
     </row>
     <row r="119">
@@ -1976,7 +1976,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1.156317830085754</v>
+        <v>1.20597767829895</v>
       </c>
     </row>
     <row r="120">
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1.112944602966309</v>
+        <v>1.18103039264679</v>
       </c>
     </row>
     <row r="121">
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1.11181914806366</v>
+        <v>1.382912158966064</v>
       </c>
     </row>
     <row r="122">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1.08794629573822</v>
+        <v>1.234981298446655</v>
       </c>
     </row>
     <row r="123">
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1.042873620986938</v>
+        <v>1.259028434753418</v>
       </c>
     </row>
     <row r="124">
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1.104063034057617</v>
+        <v>1.066580533981323</v>
       </c>
     </row>
     <row r="125">
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1.264816045761108</v>
+        <v>1.396475553512573</v>
       </c>
     </row>
     <row r="126">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>0.9868196845054626</v>
+        <v>1.061045169830322</v>
       </c>
     </row>
     <row r="127">
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1.140875577926636</v>
+        <v>1.123186111450195</v>
       </c>
     </row>
     <row r="128">
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1.111867427825928</v>
+        <v>1.062166929244995</v>
       </c>
     </row>
     <row r="129">
@@ -2106,7 +2106,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1.117970943450928</v>
+        <v>1.321682453155518</v>
       </c>
     </row>
     <row r="130">
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1.117868900299072</v>
+        <v>1.020430326461792</v>
       </c>
     </row>
     <row r="131">
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1.105257391929626</v>
+        <v>1.102832198143005</v>
       </c>
     </row>
     <row r="132">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1.104847431182861</v>
+        <v>1.105316519737244</v>
       </c>
     </row>
     <row r="133">
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1.098113059997559</v>
+        <v>1.214827656745911</v>
       </c>
     </row>
     <row r="134">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>0.9193248748779297</v>
+        <v>1.123018741607666</v>
       </c>
     </row>
     <row r="135">
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1.353787183761597</v>
+        <v>1.124219298362732</v>
       </c>
     </row>
     <row r="136">
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1.179932117462158</v>
+        <v>1.280649900436401</v>
       </c>
     </row>
     <row r="137">
@@ -2210,7 +2210,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1.286162614822388</v>
+        <v>1.251144289970398</v>
       </c>
     </row>
     <row r="138">
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1.153550267219543</v>
+        <v>1.331140041351318</v>
       </c>
     </row>
     <row r="139">
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1.089845895767212</v>
+        <v>1.196755647659302</v>
       </c>
     </row>
     <row r="140">
@@ -2249,7 +2249,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1.242084741592407</v>
+        <v>1.331754922866821</v>
       </c>
     </row>
     <row r="141">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1.019483089447021</v>
+        <v>1.288828372955322</v>
       </c>
     </row>
     <row r="142">
@@ -2275,7 +2275,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1.106335043907166</v>
+        <v>1.159123420715332</v>
       </c>
     </row>
     <row r="143">
@@ -2288,51 +2288,51 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1.168344259262085</v>
+        <v>1.163367033004761</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>142</v>
+        <v>0</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1.163205027580261</v>
+        <v>1.183721542358398</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>143</v>
+        <v>1</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1.023992896080017</v>
+        <v>1.045955657958984</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>144</v>
+        <v>2</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1.059399247169495</v>
+        <v>1.08397912979126</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -2340,12 +2340,12 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1.029006719589233</v>
+        <v>1.025399208068848</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -2353,12 +2353,12 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1.019188642501831</v>
+        <v>1.02554976940155</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -2366,12 +2366,12 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>0.9465954303741455</v>
+        <v>1.009798645973206</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -2379,12 +2379,12 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>1.270362019538879</v>
+        <v>1.085214138031006</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -2392,12 +2392,12 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1.129815816879272</v>
+        <v>1.133800506591797</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -2405,12 +2405,12 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>1.038190960884094</v>
+        <v>1.055475950241089</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -2418,12 +2418,12 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1.075128436088562</v>
+        <v>1.2667156457901</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -2431,12 +2431,12 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>1.208035945892334</v>
+        <v>1.011519908905029</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -2444,12 +2444,12 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>1.123610854148865</v>
+        <v>1.089776515960693</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -2457,12 +2457,12 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1.268611550331116</v>
+        <v>1.017474412918091</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -2470,12 +2470,12 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>1.145689725875854</v>
+        <v>1.182649493217468</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -2483,12 +2483,12 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>1.113592863082886</v>
+        <v>1.143447875976562</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -2496,12 +2496,12 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1.166638851165771</v>
+        <v>1.135980606079102</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -2509,12 +2509,12 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1.090310454368591</v>
+        <v>1.120989918708801</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -2522,12 +2522,12 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1.248677849769592</v>
+        <v>1.153409481048584</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -2535,12 +2535,12 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>1.196480512619019</v>
+        <v>1.120377063751221</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -2548,12 +2548,12 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1.178213834762573</v>
+        <v>1.12923264503479</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -2561,12 +2561,12 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1.245404481887817</v>
+        <v>1.092288732528687</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -2574,12 +2574,12 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1.064226031303406</v>
+        <v>1.089686155319214</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -2587,12 +2587,12 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1.114523649215698</v>
+        <v>1.014212608337402</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -2600,12 +2600,12 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1.10630202293396</v>
+        <v>1.063700914382935</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -2613,12 +2613,12 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1.088428378105164</v>
+        <v>1.000975728034973</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -2626,12 +2626,12 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1.202323079109192</v>
+        <v>1.106532692909241</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -2639,12 +2639,12 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1.218406915664673</v>
+        <v>1.207182645797729</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -2652,12 +2652,12 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1.111911416053772</v>
+        <v>1.04774272441864</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -2665,12 +2665,12 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1.21106219291687</v>
+        <v>1.185251235961914</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -2678,12 +2678,12 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1.114140868186951</v>
+        <v>1.236515760421753</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -2691,12 +2691,12 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1.133249044418335</v>
+        <v>1.059663534164429</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -2704,12 +2704,12 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1.068856000900269</v>
+        <v>1.019513726234436</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -2717,12 +2717,12 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1.130230188369751</v>
+        <v>1.054070472717285</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -2730,12 +2730,12 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1.072528123855591</v>
+        <v>1.159360408782959</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -2743,12 +2743,12 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1.073189735412598</v>
+        <v>1.088114619255066</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -2756,12 +2756,12 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1.115813732147217</v>
+        <v>1.083367705345154</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -2769,12 +2769,12 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1.105438590049744</v>
+        <v>1.033088564872742</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -2782,12 +2782,12 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1.112380027770996</v>
+        <v>1.227433681488037</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -2795,12 +2795,12 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1.091463327407837</v>
+        <v>1.154003620147705</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -2808,12 +2808,12 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1.076156973838806</v>
+        <v>1.285191655158997</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -2821,12 +2821,12 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1.011194944381714</v>
+        <v>1.325854182243347</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -2834,12 +2834,12 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1.066086292266846</v>
+        <v>1.263845682144165</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -2847,12 +2847,12 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1.125456809997559</v>
+        <v>1.219465017318726</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -2860,12 +2860,12 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1.06172502040863</v>
+        <v>1.169871807098389</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -2873,12 +2873,12 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1.055083155632019</v>
+        <v>1.083807229995728</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -2886,12 +2886,12 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1.253124713897705</v>
+        <v>1.029536962509155</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -2899,12 +2899,12 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1.096014976501465</v>
+        <v>1.192089200019836</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -2912,12 +2912,12 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1.102940201759338</v>
+        <v>1.223511695861816</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -2925,12 +2925,12 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1.110868215560913</v>
+        <v>1.147119045257568</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -2938,12 +2938,12 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1.247392654418945</v>
+        <v>1.129121661186218</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -2951,12 +2951,12 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1.268808364868164</v>
+        <v>1.326428174972534</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -2964,12 +2964,12 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1.156513214111328</v>
+        <v>1.135279297828674</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -2977,12 +2977,12 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1.100793600082397</v>
+        <v>1.108225345611572</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -2990,12 +2990,12 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1.094105243682861</v>
+        <v>0.9873982071876526</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -3003,12 +3003,12 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1.092611193656921</v>
+        <v>1.068362474441528</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -3016,12 +3016,12 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1.250544309616089</v>
+        <v>1.181455373764038</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -3029,12 +3029,12 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1.169813394546509</v>
+        <v>1.067682862281799</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -3042,12 +3042,12 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1.107247233390808</v>
+        <v>1.227601528167725</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -3055,12 +3055,12 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1.274910449981689</v>
+        <v>1.258273363113403</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -3068,12 +3068,12 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1.082607507705688</v>
+        <v>1.30417275428772</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -3081,12 +3081,12 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1.245035648345947</v>
+        <v>1.129448533058167</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -3094,12 +3094,12 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1.188917398452759</v>
+        <v>1.137550592422485</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -3107,12 +3107,12 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1.115910887718201</v>
+        <v>1.126591205596924</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -3120,12 +3120,12 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1.179152846336365</v>
+        <v>1.157334566116333</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -3133,12 +3133,12 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1.167362451553345</v>
+        <v>1.127120733261108</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -3146,12 +3146,12 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1.161375522613525</v>
+        <v>1.000304698944092</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -3159,12 +3159,12 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1.102116584777832</v>
+        <v>1.215262293815613</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -3172,12 +3172,12 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>1.090483427047729</v>
+        <v>1.131986618041992</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
@@ -3185,12 +3185,12 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1.103931188583374</v>
+        <v>1.008620023727417</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
@@ -3198,12 +3198,12 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1.200171828269958</v>
+        <v>1.126991510391235</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -3211,12 +3211,12 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1.247670412063599</v>
+        <v>1.213808298110962</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -3224,12 +3224,12 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1.128261089324951</v>
+        <v>1.215035915374756</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
@@ -3237,12 +3237,12 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>1.234970092773438</v>
+        <v>1.084051728248596</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -3250,12 +3250,12 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1.157668590545654</v>
+        <v>1.264666199684143</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -3263,12 +3263,12 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1.057155966758728</v>
+        <v>1.02496063709259</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -3276,12 +3276,12 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1.183168292045593</v>
+        <v>1.11652934551239</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -3289,12 +3289,12 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1.099884748458862</v>
+        <v>1.256845593452454</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -3302,12 +3302,12 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1.185989618301392</v>
+        <v>1.078456878662109</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -3315,12 +3315,12 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1.227895975112915</v>
+        <v>1.103941440582275</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -3328,12 +3328,12 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1.11573588848114</v>
+        <v>1.040603041648865</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -3341,12 +3341,12 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1.122878670692444</v>
+        <v>1.000349283218384</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -3354,12 +3354,12 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1.191376924514771</v>
+        <v>1.182228803634644</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -3367,12 +3367,12 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1.238003253936768</v>
+        <v>1.177301049232483</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -3380,12 +3380,12 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1.102315783500671</v>
+        <v>1.075261950492859</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -3393,12 +3393,12 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1.079561352729797</v>
+        <v>1.096480846405029</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -3406,12 +3406,12 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1.017154097557068</v>
+        <v>1.311904668807983</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -3419,12 +3419,12 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1.142343521118164</v>
+        <v>1.038891553878784</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -3432,12 +3432,12 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1.168028831481934</v>
+        <v>1.038293361663818</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
@@ -3445,12 +3445,12 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1.113789558410645</v>
+        <v>1.037760734558105</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -3458,12 +3458,12 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1.049837708473206</v>
+        <v>1.035258173942566</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -3471,12 +3471,12 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1.320904016494751</v>
+        <v>1.138743758201599</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -3484,12 +3484,12 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1.227337837219238</v>
+        <v>0.9794855713844299</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
@@ -3497,12 +3497,12 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1.154294013977051</v>
+        <v>1.256964445114136</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
@@ -3510,12 +3510,12 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1.227082133293152</v>
+        <v>1.103139162063599</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
@@ -3523,12 +3523,12 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1.231560468673706</v>
+        <v>1.050968170166016</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
@@ -3536,12 +3536,12 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1.095353722572327</v>
+        <v>1.108479499816895</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
@@ -3549,12 +3549,12 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1.123173594474792</v>
+        <v>1.02675199508667</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
@@ -3562,12 +3562,12 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1.026131272315979</v>
+        <v>1.179380297660828</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
@@ -3575,12 +3575,12 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1.131212949752808</v>
+        <v>1.149889230728149</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
@@ -3588,12 +3588,12 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1.109793424606323</v>
+        <v>1.059972047805786</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
@@ -3601,12 +3601,12 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1.081534862518311</v>
+        <v>1.239729881286621</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
@@ -3614,12 +3614,12 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1.196480751037598</v>
+        <v>1.147481560707092</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
@@ -3627,12 +3627,12 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1.056267976760864</v>
+        <v>1.154932975769043</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
@@ -3640,12 +3640,12 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1.142531871795654</v>
+        <v>1.09272837638855</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
@@ -3653,12 +3653,12 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1.200705885887146</v>
+        <v>1.080776214599609</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
@@ -3666,12 +3666,12 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1.141160011291504</v>
+        <v>1.46975040435791</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B250" t="inlineStr">
         <is>
@@ -3679,12 +3679,12 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1.057660102844238</v>
+        <v>1.123306035995483</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B251" t="inlineStr">
         <is>
@@ -3692,12 +3692,12 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1.211716890335083</v>
+        <v>1.18469762802124</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B252" t="inlineStr">
         <is>
@@ -3705,12 +3705,12 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1.188100814819336</v>
+        <v>1.075399398803711</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B253" t="inlineStr">
         <is>
@@ -3718,12 +3718,12 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>0.9754804372787476</v>
+        <v>1.120050668716431</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
@@ -3731,12 +3731,12 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1.176705598831177</v>
+        <v>1.109665751457214</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
@@ -3744,12 +3744,12 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1.144629716873169</v>
+        <v>1.036745548248291</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
@@ -3757,12 +3757,12 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1.236431360244751</v>
+        <v>1.018447637557983</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
@@ -3770,12 +3770,12 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>1.150770425796509</v>
+        <v>1.082565069198608</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
@@ -3783,12 +3783,12 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>1.244355916976929</v>
+        <v>1.231321692466736</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
@@ -3796,12 +3796,12 @@
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1.199227333068848</v>
+        <v>1.129101037979126</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B260" t="inlineStr">
         <is>
@@ -3809,12 +3809,12 @@
         </is>
       </c>
       <c r="C260" t="n">
-        <v>0.94748854637146</v>
+        <v>1.045676112174988</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B261" t="inlineStr">
         <is>
@@ -3822,12 +3822,12 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1.061436176300049</v>
+        <v>1.065483093261719</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B262" t="inlineStr">
         <is>
@@ -3835,12 +3835,12 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1.204064130783081</v>
+        <v>1.145095705986023</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B263" t="inlineStr">
         <is>
@@ -3848,12 +3848,12 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1.183825492858887</v>
+        <v>1.19810938835144</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B264" t="inlineStr">
         <is>
@@ -3861,12 +3861,12 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1.267158269882202</v>
+        <v>1.225695133209229</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B265" t="inlineStr">
         <is>
@@ -3874,12 +3874,12 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1.083116769790649</v>
+        <v>1.03121030330658</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B266" t="inlineStr">
         <is>
@@ -3887,12 +3887,12 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1.124401688575745</v>
+        <v>1.115338325500488</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B267" t="inlineStr">
         <is>
@@ -3900,12 +3900,12 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1.124760389328003</v>
+        <v>1.103427767753601</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B268" t="inlineStr">
         <is>
@@ -3913,12 +3913,12 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>1.045652270317078</v>
+        <v>1.165964603424072</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B269" t="inlineStr">
         <is>
@@ -3926,12 +3926,12 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>1.122270941734314</v>
+        <v>1.088280558586121</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
@@ -3939,12 +3939,12 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>1.121262550354004</v>
+        <v>1.239283800125122</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
@@ -3952,12 +3952,12 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1.100843667984009</v>
+        <v>0.9706224203109741</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
@@ -3965,12 +3965,12 @@
         </is>
       </c>
       <c r="C272" t="n">
-        <v>1.109004735946655</v>
+        <v>1.346990585327148</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
@@ -3978,12 +3978,12 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>1.102344036102295</v>
+        <v>1.137148141860962</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
@@ -3991,12 +3991,12 @@
         </is>
       </c>
       <c r="C274" t="n">
-        <v>1.100701332092285</v>
+        <v>1.041587471961975</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
@@ -4004,12 +4004,12 @@
         </is>
       </c>
       <c r="C275" t="n">
-        <v>1.104910850524902</v>
+        <v>1.14850902557373</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
@@ -4017,12 +4017,12 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>1.14866030216217</v>
+        <v>1.126264095306396</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
@@ -4030,12 +4030,12 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>1.297993898391724</v>
+        <v>1.196461200714111</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
@@ -4043,12 +4043,12 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>0.9454213380813599</v>
+        <v>1.07879626750946</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
@@ -4056,12 +4056,12 @@
         </is>
       </c>
       <c r="C279" t="n">
-        <v>1.160290241241455</v>
+        <v>1.273513555526733</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
@@ -4069,12 +4069,12 @@
         </is>
       </c>
       <c r="C280" t="n">
-        <v>1.223099946975708</v>
+        <v>1.111710786819458</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
@@ -4082,12 +4082,12 @@
         </is>
       </c>
       <c r="C281" t="n">
-        <v>1.251889228820801</v>
+        <v>1.150387287139893</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
@@ -4095,12 +4095,12 @@
         </is>
       </c>
       <c r="C282" t="n">
-        <v>1.220222473144531</v>
+        <v>1.228474140167236</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
@@ -4108,12 +4108,12 @@
         </is>
       </c>
       <c r="C283" t="n">
-        <v>1.167181730270386</v>
+        <v>1.15317714214325</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
@@ -4121,12 +4121,12 @@
         </is>
       </c>
       <c r="C284" t="n">
-        <v>1.128097772598267</v>
+        <v>1.316272258758545</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
@@ -4134,12 +4134,12 @@
         </is>
       </c>
       <c r="C285" t="n">
-        <v>1.085383296012878</v>
+        <v>1.200599193572998</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
@@ -4147,12 +4147,12 @@
         </is>
       </c>
       <c r="C286" t="n">
-        <v>1.064168214797974</v>
+        <v>1.038123488426208</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
@@ -4160,12 +4160,12 @@
         </is>
       </c>
       <c r="C287" t="n">
-        <v>1.071036100387573</v>
+        <v>1.017375946044922</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
@@ -4173,46 +4173,7 @@
         </is>
       </c>
       <c r="C288" t="n">
-        <v>1.212243676185608</v>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="n">
-        <v>142</v>
-      </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C289" t="n">
-        <v>1.167740702629089</v>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="n">
-        <v>143</v>
-      </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C290" t="n">
-        <v>0.9969061613082886</v>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="n">
-        <v>144</v>
-      </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C291" t="n">
-        <v>1.028416633605957</v>
+        <v>1.02042555809021</v>
       </c>
     </row>
   </sheetData>

</xml_diff>